<commit_message>
chore(preview): TTE.PA outputs regeneres
</commit_message>
<xml_diff>
--- a/preview/TTE.PA/TTE.PA_financials.xlsx
+++ b/preview/TTE.PA/TTE.PA_financials.xlsx
@@ -8039,10 +8039,18 @@
         </is>
       </c>
       <c r="D29" s="266" t="n"/>
-      <c r="E29" s="266" t="n"/>
-      <c r="F29" s="266" t="n"/>
-      <c r="G29" s="266" t="n"/>
-      <c r="H29" s="266" t="n"/>
+      <c r="E29" s="266" t="n">
+        <v>-1823</v>
+      </c>
+      <c r="F29" s="266" t="n">
+        <v>-7711</v>
+      </c>
+      <c r="G29" s="266" t="n">
+        <v>-9167</v>
+      </c>
+      <c r="H29" s="266" t="n">
+        <v>-7995</v>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="3" t="n"/>
@@ -9085,10 +9093,18 @@
         </is>
       </c>
       <c r="D79" s="266" t="n"/>
-      <c r="E79" s="266" t="n"/>
-      <c r="F79" s="266" t="n"/>
-      <c r="G79" s="266" t="n"/>
-      <c r="H79" s="266" t="n"/>
+      <c r="E79" s="266" t="n">
+        <v>722</v>
+      </c>
+      <c r="F79" s="266" t="n">
+        <v>577</v>
+      </c>
+      <c r="G79" s="266" t="n">
+        <v>490</v>
+      </c>
+      <c r="H79" s="266" t="n">
+        <v>347</v>
+      </c>
     </row>
     <row r="80" ht="15" customHeight="1" thickBot="1">
       <c r="A80" s="3" t="n"/>
@@ -9417,7 +9433,7 @@
       <c r="F95" s="266" t="n"/>
       <c r="G95" s="266" t="n"/>
       <c r="H95" s="266" t="n">
-        <v>79.09</v>
+        <v>78.48999999999999</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1">
@@ -9543,7 +9559,7 @@
       <c r="F100" s="266" t="n"/>
       <c r="G100" s="266" t="n"/>
       <c r="H100" s="266" t="n">
-        <v>0.0442</v>
+        <v>0.0444</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1">
@@ -9611,7 +9627,7 @@
       <c r="F103" s="266" t="n"/>
       <c r="G103" s="266" t="n"/>
       <c r="H103" s="266" t="n">
-        <v>0.0592</v>
+        <v>0.0594</v>
       </c>
     </row>
     <row r="104" ht="15" customHeight="1">
@@ -9953,7 +9969,7 @@
       </c>
       <c r="D120" s="272" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="E120" s="273" t="n"/>
@@ -10376,7 +10392,7 @@
         </is>
       </c>
       <c r="C14" s="536" t="n">
-        <v>79.09</v>
+        <v>78.48999999999999</v>
       </c>
     </row>
     <row r="15">
@@ -20392,10 +20408,10 @@
         </is>
       </c>
       <c r="D9" s="477" t="n">
-        <v>165.43</v>
+        <v>170.99</v>
       </c>
       <c r="E9" s="36" t="n">
-        <v>736353.65</v>
+        <v>759520.89</v>
       </c>
       <c r="F9" s="36" t="n">
         <v>323905</v>
@@ -20433,10 +20449,10 @@
         </is>
       </c>
       <c r="D10" s="477" t="n">
-        <v>3472.5</v>
+        <v>3482</v>
       </c>
       <c r="E10" s="36" t="n">
-        <v>242993.27</v>
+        <v>243531.1</v>
       </c>
       <c r="F10" s="36" t="n">
         <v>266886</v>
@@ -20454,7 +20470,7 @@
       </c>
       <c r="J10" s="479" t="n"/>
       <c r="K10" s="477" t="n">
-        <v>2.23</v>
+        <v>2.25</v>
       </c>
       <c r="L10" s="478">
         <f>IFERROR(D10/K10,"–")</f>
@@ -20474,10 +20490,10 @@
         </is>
       </c>
       <c r="D11" s="477" t="n">
-        <v>583.1</v>
+        <v>584.1</v>
       </c>
       <c r="E11" s="36" t="n">
-        <v>146505.68</v>
+        <v>146659.44</v>
       </c>
       <c r="F11" s="36" t="n">
         <v>187637.01</v>
@@ -20513,10 +20529,10 @@
         </is>
       </c>
       <c r="D12" s="477" t="n">
-        <v>23.64</v>
+        <v>23.93</v>
       </c>
       <c r="E12" s="36" t="n">
-        <v>93486.88</v>
+        <v>94325.11</v>
       </c>
       <c r="F12" s="36" t="n">
         <v>83604</v>
@@ -20554,10 +20570,10 @@
         </is>
       </c>
       <c r="D13" s="480" t="n">
-        <v>24.17</v>
+        <v>24.07</v>
       </c>
       <c r="E13" s="71" t="n">
-        <v>34329.25</v>
+        <v>34218.74</v>
       </c>
       <c r="F13" s="71" t="n">
         <v>48349</v>

</xml_diff>